<commit_message>
Updated cure data (v50)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_cure.xlsx
+++ b/src/data/routekaart_status_cure.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561EBB31-AF43-42C0-82B3-0EBC8A1914EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD86D89A-1F18-4694-8543-F33E155EC79A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="1520" windowWidth="31120" windowHeight="19700" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="13660" yWindow="1770" windowWidth="22740" windowHeight="13990" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="79">
   <si>
     <t>Amsterdam UMC</t>
   </si>
@@ -257,6 +257,15 @@
   </si>
   <si>
     <t>Medisch Centrum Leeuwarden</t>
+  </si>
+  <si>
+    <t>Kentalis</t>
+  </si>
+  <si>
+    <t>Rijndam Revalidatie</t>
+  </si>
+  <si>
+    <t>Saxenburgh Groep</t>
   </si>
 </sst>
 </file>
@@ -617,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.7265625" customWidth="1"/>
@@ -834,7 +843,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
         <v>24</v>
@@ -842,7 +851,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="B28" t="s">
         <v>24</v>
@@ -850,7 +859,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
         <v>24</v>
@@ -858,7 +867,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
         <v>24</v>
@@ -866,7 +875,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="B31" t="s">
         <v>24</v>
@@ -874,7 +883,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B32" t="s">
         <v>24</v>
@@ -882,7 +891,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
         <v>24</v>
@@ -890,7 +899,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B34" t="s">
         <v>24</v>
@@ -898,7 +907,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="B35" t="s">
         <v>24</v>
@@ -906,7 +915,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B36" t="s">
         <v>24</v>
@@ -914,7 +923,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
         <v>24</v>
@@ -922,7 +931,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="B38" t="s">
         <v>24</v>
@@ -930,7 +939,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
         <v>24</v>
@@ -938,7 +947,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="B40" t="s">
         <v>24</v>
@@ -946,7 +955,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B41" t="s">
         <v>24</v>
@@ -954,7 +963,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="B42" t="s">
         <v>24</v>
@@ -962,7 +971,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B43" t="s">
         <v>24</v>
@@ -970,7 +979,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B44" t="s">
         <v>24</v>
@@ -978,23 +987,23 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B46" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="B47" t="s">
         <v>24</v>
@@ -1002,7 +1011,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B48" t="s">
         <v>24</v>
@@ -1010,7 +1019,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="B49" t="s">
         <v>24</v>
@@ -1018,15 +1027,15 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B50" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B51" t="s">
         <v>24</v>
@@ -1034,7 +1043,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B52" t="s">
         <v>24</v>
@@ -1042,7 +1051,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="B53" t="s">
         <v>24</v>
@@ -1050,7 +1059,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B54" t="s">
         <v>24</v>
@@ -1058,7 +1067,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B55" t="s">
         <v>24</v>
@@ -1066,7 +1075,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B56" t="s">
         <v>24</v>
@@ -1074,7 +1083,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B57" t="s">
         <v>24</v>
@@ -1082,7 +1091,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="B58" t="s">
         <v>24</v>
@@ -1090,7 +1099,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="B59" t="s">
         <v>24</v>
@@ -1098,7 +1107,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B60" t="s">
         <v>24</v>
@@ -1106,7 +1115,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="B61" t="s">
         <v>24</v>
@@ -1114,7 +1123,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B62" t="s">
         <v>24</v>
@@ -1122,7 +1131,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="B63" t="s">
         <v>24</v>
@@ -1130,7 +1139,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B64" t="s">
         <v>24</v>
@@ -1138,7 +1147,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B65" t="s">
         <v>24</v>
@@ -1146,7 +1155,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B66" t="s">
         <v>24</v>
@@ -1154,7 +1163,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B67" t="s">
         <v>24</v>
@@ -1162,15 +1171,15 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="B68" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="B69" t="s">
         <v>24</v>
@@ -1178,7 +1187,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B70" t="s">
         <v>24</v>
@@ -1186,15 +1195,15 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="B71" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="B72" t="s">
         <v>24</v>
@@ -1202,9 +1211,33 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>36</v>
+      </c>
+      <c r="B73" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>63</v>
+      </c>
+      <c r="B74" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>71</v>
+      </c>
+      <c r="B75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>57</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B76" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>